<commit_message>
Fix question import templates and SQL test cases
</commit_message>
<xml_diff>
--- a/examples/import/example_questions.xlsx
+++ b/examples/import/example_questions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:Y6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -460,13 +460,28 @@
       <c r="T1" t="str">
         <v>output_format</v>
       </c>
+      <c r="U1" t="str">
+        <v>schema_sql</v>
+      </c>
+      <c r="V1" t="str">
+        <v>sample_data_sql</v>
+      </c>
+      <c r="W1" t="str">
+        <v>sample_expected_output</v>
+      </c>
+      <c r="X1" t="str">
+        <v>order_sensitive</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>test_cases</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>mcq</v>
       </c>
       <c r="B2" t="str">
-        <v>What is the time complexity of searching in a balanced BST?</v>
+        <v>Phani is cleaning a dataset in Pandas. Which method should he use to remove all rows containing at least one NaN value?</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -475,7 +490,7 @@
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>Easy</v>
+        <v>Medium</v>
       </c>
       <c r="F2">
         <v>2</v>
@@ -484,19 +499,19 @@
         <v>0.5</v>
       </c>
       <c r="H2" t="str">
-        <v>In a balanced BST with N nodes, the height is O(log N).</v>
+        <v>The dropna() method removes missing values (NaN) from a DataFrame.</v>
       </c>
       <c r="I2" t="str">
-        <v>O(log N)</v>
+        <v>df.dropna()</v>
       </c>
       <c r="J2" t="str">
-        <v>O(N)</v>
+        <v>df.fillna()</v>
       </c>
       <c r="K2" t="str">
-        <v>O(1)</v>
+        <v>df.remove_nan()</v>
       </c>
       <c r="L2" t="str">
-        <v>O(N log N)</v>
+        <v>df.drop_null()</v>
       </c>
       <c r="M2" t="str">
         <v>A</v>
@@ -520,6 +535,21 @@
         <v/>
       </c>
       <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
         <v/>
       </c>
     </row>
@@ -528,7 +558,7 @@
         <v>mcq</v>
       </c>
       <c r="B3" t="str">
-        <v>Which of the following data structures operates on a First-In-First-Out (FIFO) basis?</v>
+        <v>Sarva anna is analyzing sales data in SQL. Which clause should he use to filter the results of an aggregation like COUNT() &gt; 5?</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -543,22 +573,22 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H3" t="str">
-        <v>A Queue processes elements in FIFO order.</v>
+        <v>The HAVING clause is used to filter groups based on aggregate functions.</v>
       </c>
       <c r="I3" t="str">
-        <v>Queue</v>
+        <v>HAVING</v>
       </c>
       <c r="J3" t="str">
-        <v>Stack</v>
+        <v>WHERE</v>
       </c>
       <c r="K3" t="str">
-        <v>Binary Tree</v>
+        <v>FILTER</v>
       </c>
       <c r="L3" t="str">
-        <v>Priority Queue</v>
+        <v>GROUP BY</v>
       </c>
       <c r="M3" t="str">
         <v>A</v>
@@ -582,74 +612,264 @@
         <v/>
       </c>
       <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>coding</v>
+        <v>mcq</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>Raghavi is using Excel to look up a value in the leftmost column of a table. Which function is most appropriate?</v>
       </c>
       <c r="C4" t="str">
-        <v>Two Sum Problem</v>
+        <v/>
       </c>
       <c r="D4" t="str">
-        <v>Given two space-separated integers A and B on standard input, output their sum (A + B).</v>
+        <v/>
       </c>
       <c r="E4" t="str">
         <v>Easy</v>
       </c>
       <c r="F4">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>VLOOKUP searches for a value in the first column of a table array and returns a value in the same row from another column.</v>
       </c>
       <c r="I4" t="str">
-        <v/>
+        <v>VLOOKUP</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>HLOOKUP</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>MATCH</v>
       </c>
       <c r="L4" t="str">
-        <v/>
+        <v>INDEX</v>
       </c>
       <c r="M4" t="str">
-        <v/>
+        <v>A</v>
       </c>
       <c r="N4" t="str">
-        <v>4 7</v>
+        <v/>
       </c>
       <c r="O4" t="str">
-        <v>11</v>
+        <v/>
       </c>
       <c r="P4" t="str">
-        <v>100 200</v>
+        <v/>
       </c>
       <c r="Q4" t="str">
-        <v>300</v>
+        <v/>
       </c>
       <c r="R4" t="str">
-        <v>-10^9 &lt;= A, B &lt;= 10^9</v>
+        <v/>
       </c>
       <c r="S4" t="str">
-        <v>Two integers A and B separated by space.</v>
+        <v/>
       </c>
       <c r="T4" t="str">
-        <v>Single integer A + B.</v>
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>coding</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v>Data Guide Python Challenge</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Srishanth wants to find the sum of all elements in an array of integers that are strictly greater than the array's average. Write a program to help him.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F5">
+        <v>10</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str" xml:space="preserve">
+        <v xml:space="preserve">5
+10 20 30 40 50</v>
+      </c>
+      <c r="O5" t="str">
+        <v>90</v>
+      </c>
+      <c r="P5" t="str" xml:space="preserve">
+        <v xml:space="preserve">4
+-5 10 15 20</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>35</v>
+      </c>
+      <c r="R5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1 &lt;= N &lt;= 10^5
+-1000 &lt;= array[i] &lt;= 1000</v>
+      </c>
+      <c r="S5" t="str" xml:space="preserve">
+        <v xml:space="preserve">The first line contains N, the number of elements.
+The second line contains N space-separated integers.</v>
+      </c>
+      <c r="T5" t="str">
+        <v>A single integer denoting the sum of elements greater than the average.</v>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v>[{"input":"5\n10 20 30 40 50","expected_output":"90","is_sample":true,"is_hidden":false,"weight":1},{"input":"4\n-5 10 15 20","expected_output":"35","is_sample":false,"is_hidden":true,"weight":2}]</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>sql</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v>Kaushik Anna's Tech Store</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Kaushik anna wants a list of all products in his store that cost more than $50.00, sorted by price in descending order. Write the SQL query to retrieve the name and price.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v>CREATE TABLE products (id INTEGER PRIMARY KEY, name TEXT NOT NULL, price REAL NOT NULL, category TEXT);</v>
+      </c>
+      <c r="V6" t="str">
+        <v>INSERT INTO products VALUES (1, 'Mechanical Keyboard', 120.50, 'Electronics'), (2, 'Mousepad', 15.00, 'Accessories'), (3, 'Wireless Mouse', 65.00, 'Electronics');</v>
+      </c>
+      <c r="W6" t="str" xml:space="preserve">
+        <v xml:space="preserve">name | price
+Mechanical Keyboard | 120.5
+Wireless Mouse | 65.0</v>
+      </c>
+      <c r="X6" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y6" t="str">
+        <v>[{"setup_sql":"INSERT INTO products VALUES (1, 'Mechanical Keyboard', 120.50, 'Electronics'), (2, 'Mousepad', 15.00, 'Accessories'), (3, 'Wireless Mouse', 65.00, 'Electronics');","expected_output":"name | price\nMechanical Keyboard | 120.5\nWireless Mouse | 65.0","is_sample":true,"is_hidden":false,"weight":1},{"setup_sql":"INSERT INTO products VALUES (1, 'Mechanical Keyboard', 120.50, 'Electronics'), (2, 'Mousepad', 15.00, 'Accessories'), (3, 'Wireless Mouse', 65.00, 'Electronics'), (4, 'Monitor', 300.00, 'Electronics');","expected_output":"name | price\nMonitor | 300.0\nMechanical Keyboard | 120.5\nWireless Mouse | 65.0","is_sample":false,"is_hidden":true,"weight":2}]</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>